<commit_message>
changes in leave TC.
</commit_message>
<xml_diff>
--- a/Data Files/excel.xlsx
+++ b/Data Files/excel.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Diksha Thakur\Katalon Studio\katalondemo\myfirstKatalonProject\Data Files\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B2C084E-1014-49EA-81D1-7C500A93AC1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="60" windowWidth="20115" windowHeight="8010" activeTab="2"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -16,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="28">
   <si>
     <t>Url</t>
   </si>
@@ -96,13 +102,16 @@
     <t>Diksha Thakur</t>
   </si>
   <si>
-    <t>2025/14/05</t>
+    <t>2025-14-05</t>
+  </si>
+  <si>
+    <t>2025-15-05</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -156,14 +165,17 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
   </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -201,7 +213,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -273,7 +285,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -446,7 +458,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -484,7 +496,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -537,8 +549,8 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="E2" r:id="rId1"/>
-    <hyperlink ref="F2" r:id="rId2"/>
+    <hyperlink ref="E2" r:id="rId1" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
+    <hyperlink ref="F2" r:id="rId2" xr:uid="{00000000-0004-0000-0100-000001000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId3"/>
@@ -546,7 +558,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -585,8 +597,8 @@
       <c r="A2" t="s">
         <v>26</v>
       </c>
-      <c r="B2" s="2">
-        <v>45662</v>
+      <c r="B2" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="C2" t="s">
         <v>19</v>

</xml_diff>

<commit_message>
FEAT : Added read and write code for excel.
</commit_message>
<xml_diff>
--- a/Data Files/excel.xlsx
+++ b/Data Files/excel.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28730"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Diksha Thakur\Katalon Studio\katalondemo\myfirstKatalonProject\Data Files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B2C084E-1014-49EA-81D1-7C500A93AC1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52D0B560-E090-49BD-B654-77CE9F362B66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -102,10 +102,10 @@
     <t>Diksha Thakur</t>
   </si>
   <si>
-    <t>2025-14-05</t>
-  </si>
-  <si>
     <t>2025-15-05</t>
+  </si>
+  <si>
+    <t>2025-16-05</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
FIX : Done changes like renaming,use encrypted password.
</commit_message>
<xml_diff>
--- a/Data Files/excel.xlsx
+++ b/Data Files/excel.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Diksha Thakur\Katalon Studio\katalondemo\myfirstKatalonProject\Data Files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52D0B560-E090-49BD-B654-77CE9F362B66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99F33A5C-A515-44FC-B5EC-2B91CD6F8147}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2550" yWindow="2550" windowWidth="15375" windowHeight="7875" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="admin" sheetId="2" r:id="rId2"/>
     <sheet name="leave" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="144525"/>
@@ -84,9 +84,6 @@
     <t>Taken</t>
   </si>
   <si>
-    <t>CAN- Personal</t>
-  </si>
-  <si>
     <t>leaveType</t>
   </si>
   <si>
@@ -106,6 +103,9 @@
   </si>
   <si>
     <t>2025-16-05</t>
+  </si>
+  <si>
+    <t>CAN - Bereavement</t>
   </si>
 </sst>
 </file>
@@ -584,33 +584,33 @@
         <v>18</v>
       </c>
       <c r="D1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F1" t="s">
         <v>21</v>
-      </c>
-      <c r="E1" t="s">
-        <v>24</v>
-      </c>
-      <c r="F1" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>26</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>27</v>
       </c>
       <c r="C2" t="s">
         <v>19</v>
       </c>
       <c r="D2" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="E2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>